<commit_message>
Crawlability audit: fixes from verification pass (rate-limit rows, Leumit robots/sitemap, verified 301 targets, counts)
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/crawlability-admati-september-2026.xlsx
+++ b/public/crawlability-admati-september-2026.xlsx
@@ -547,7 +547,7 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>להריץ מחדש את ה-Website Audit של admati ב-SE Ranking (הסריקה האחרונה: 2024-04-14).</t>
+          <t>להריץ מחדש את ה-Website Audit של admati ב-SE Ranking (הסריקה האחרונה: 2024-04-14); הפעלה מחדש דרך ה-API אינה זמינה בחשבון, יש להפעיל בממשק.</t>
         </is>
       </c>
     </row>
@@ -668,7 +668,7 @@
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>לתקן או להסיר את הקישור בעמודי המקור; להגדיר הפניית 301 ליעד המצוין. יעד משוער לפי הקטגוריה הקרובה; לאישור.</t>
+          <t>לתקן או להסיר את הקישור בעמודי המקור. יעד מוצע להפניית 301 (אומת כעמוד תקין), לאישור הלקוח. יעד משוער לפי הקטגוריה הקרובה; לאישור.</t>
         </is>
       </c>
       <c r="J2" s="6" t="inlineStr">
@@ -715,7 +715,7 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>לתקן או להסיר את הקישור בעמודי המקור; להגדיר הפניית 301 ליעד המצוין. קטגוריית Pogo Pins בעברית קיימת בכתובת עם הסיומת -he.</t>
+          <t>לתקן או להסיר את הקישור בעמודי המקור. להגדיר הפניית 301 ליעד המצוין (אומת כעמוד תקין ב-27.09.2026). קטגוריית Pogo Pins בעברית קיימת בכתובת עם הסיומת -he.</t>
         </is>
       </c>
       <c r="J3" s="6" t="inlineStr">

</xml_diff>

<commit_message>
Crawlability audit: lean layout, findings and actions only
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/crawlability-admati-september-2026.xlsx
+++ b/public/crawlability-admati-september-2026.xlsx
@@ -502,7 +502,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>כתובות שבורות (404): 2 כתובות (הבולטת: https://admati.com/he/electromechanical/, קישור נכנס אחד). ראו פירוט בטבלה ובקובץ ה-Excel.</t>
+          <t>כתובות שבורות (404): 2 כתובות; הבולטת https://admati.com/he/electromechanical/ (קישור נכנס אחד).</t>
         </is>
       </c>
     </row>
@@ -517,7 +517,7 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>קישורים פנימיים לכתובות שמפנות (301/308): 5 כתובות (הבולטת: https://admati.com/about-he/, 276 קישורים נכנסים). ראו פירוט בטבלה ובקובץ ה-Excel.</t>
+          <t>קישורים פנימיים לכתובות שמפנות (301/308): 5 כתובות; הבולטת https://admati.com/about-he/ (276 קישורים נכנסים).</t>
         </is>
       </c>
     </row>
@@ -532,7 +532,7 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>קישורים פנימיים ללא לוכסן סופי: 2 כתובות (הבולטת: https://admati.com/he/products/laser-micromachining-2, קישור נכנס אחד). ראו פירוט בטבלה ובקובץ ה-Excel.</t>
+          <t>קישורים פנימיים ללא לוכסן סופי: 2 כתובות; הבולטת https://admati.com/he/products/laser-micromachining-2 (קישור נכנס אחד).</t>
         </is>
       </c>
     </row>
@@ -547,7 +547,7 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>להריץ מחדש את ה-Website Audit של admati ב-SE Ranking (הסריקה האחרונה: 2024-04-14); הפעלה מחדש דרך ה-API אינה זמינה בחשבון, יש להפעיל בממשק.</t>
+          <t>להריץ מחדש (בממשק) את ה-Website Audit של admati ב-SE Ranking; הסריקה האחרונה: 2024-04-14.</t>
         </is>
       </c>
     </row>
@@ -715,7 +715,7 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>לתקן או להסיר את הקישור בעמודי המקור. להגדיר הפניית 301 ליעד המצוין (אומת כעמוד תקין ב-27.09.2026). קטגוריית Pogo Pins בעברית קיימת בכתובת עם הסיומת -he.</t>
+          <t>לתקן או להסיר את הקישור בעמודי המקור. להגדיר הפניית 301 ליעד המצוין (היעד אומת כעמוד תקין). קטגוריית Pogo Pins בעברית קיימת בכתובת עם הסיומת -he.</t>
         </is>
       </c>
       <c r="J3" s="6" t="inlineStr">

</xml_diff>

<commit_message>
Crawlability audit: senior review fixes (subdomain first-hop reclassification, priorities, wording)
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/crawlability-admati-september-2026.xlsx
+++ b/public/crawlability-admati-september-2026.xlsx
@@ -466,7 +466,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:C4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -533,21 +533,6 @@
       <c r="C4" s="2" t="inlineStr">
         <is>
           <t>קישורים פנימיים ללא לוכסן סופי: 2 כתובות; הבולטת https://admati.com/he/products/laser-micromachining-2 (קישור נכנס אחד).</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="B5" s="5" t="inlineStr">
-        <is>
-          <t>נמוכה</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>להריץ מחדש (בממשק) את ה-Website Audit של admati ב-SE Ranking; הסריקה האחרונה: 2024-04-14.</t>
         </is>
       </c>
     </row>

</xml_diff>